<commit_message>
modify to ensure owner second injection assumption is displayed
</commit_message>
<xml_diff>
--- a/data/financial_projections_final.xlsx
+++ b/data/financial_projections_final.xlsx
@@ -216,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -282,6 +282,15 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -559,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -855,7 +864,7 @@
           <t>Salary expense per operating car (monthly)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="24" t="n">
         <v>3000</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1015,8 +1024,8 @@
           <t>Bank monthly instalment (principal + interest)</t>
         </is>
       </c>
-      <c r="B25" s="11">
-        <f>-PMT(B27,B26,B18)</f>
+      <c r="B25" s="25">
+        <f>-PMT(B32,B31,B23)</f>
         <v/>
       </c>
       <c r="C25" s="22" t="inlineStr">
@@ -1075,7 +1084,7 @@
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
         <is>
-          <t>Owner injection month (operating month index)</t>
+          <t>Owner second injection month (operating month index)</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
@@ -1158,8 +1167,8 @@
           <t>Bank monthly interest rate</t>
         </is>
       </c>
-      <c r="B32" s="7">
-        <f>B21/12</f>
+      <c r="B32" s="26">
+        <f>B26/12</f>
         <v/>
       </c>
       <c r="C32" s="22" t="inlineStr">
@@ -1216,81 +1225,38 @@
     <row r="35">
       <c r="A35" s="22" t="inlineStr">
         <is>
-          <t>Investor monthly payout per N$250,000 tranche</t>
+          <t>Batch 1 investor payout start month</t>
         </is>
       </c>
-      <c r="B35" s="5">
-        <f>ROUND(($B$17/$B$4)*$B$29,0)</f>
-        <v/>
+      <c r="B35" s="8" t="n">
+        <v>1</v>
       </c>
       <c r="C35" s="22" t="inlineStr">
         <is>
-          <t>N$ / month</t>
+          <t>month #</t>
         </is>
       </c>
       <c r="D35" s="22" t="inlineStr">
         <is>
-          <t>Calculated as cars funded per tranche x N$3,000 per car.</t>
+          <t>Payouts begin once the cars funded by the second owner/investor tranche start operating.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>Monthly operating profit per car</t>
+          <t>Batch 2 investor payout start month</t>
         </is>
       </c>
-      <c r="B36" s="5">
-        <f>B5-B13</f>
-        <v/>
+      <c r="B36" s="27" t="n">
+        <v>8</v>
       </c>
       <c r="C36" s="22" t="inlineStr">
-        <is>
-          <t>N$ / car / month</t>
-        </is>
-      </c>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>Calculated = gross revenue less total operating expenses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="22" t="inlineStr">
-        <is>
-          <t>Batch 1 investor payout start month</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="22" t="inlineStr">
         <is>
           <t>month #</t>
         </is>
       </c>
-      <c r="D37" s="22" t="inlineStr">
-        <is>
-          <t>Payouts begin once the cars funded by the second owner/investor tranche start operating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="22" t="inlineStr">
-        <is>
-          <t>Batch 2 investor payout start month</t>
-        </is>
-      </c>
-      <c r="B38" s="8">
-        <f>$B$23+$B$7</f>
-        <v/>
-      </c>
-      <c r="C38" s="22" t="inlineStr">
-        <is>
-          <t>month #</t>
-        </is>
-      </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Payouts begin once the cars funded by the second owner/investor tranche start operating.</t>
         </is>
@@ -17517,11 +17483,11 @@
           <t>Prime-linked amortising bank facility: N$250,000 at 10.00% p.a. over 54 months, with payments starting in operating month 5. Opening balance includes the draw in the first loan month.</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="26" t="n"/>
+      <c r="B2" s="28" t="n"/>
+      <c r="C2" s="28" t="n"/>
+      <c r="D2" s="28" t="n"/>
+      <c r="E2" s="28" t="n"/>
+      <c r="F2" s="29" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">

</xml_diff>